<commit_message>
Add manual paper watch report
</commit_message>
<xml_diff>
--- a/web/reports/monthly-top-psychology-journal-watch/2026-07_all.xlsx
+++ b/web/reports/monthly-top-psychology-journal-watch/2026-07_all.xlsx
@@ -55,22 +55,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>governance_society</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Publisher Correction: Happiness and Single Parenthood: A Literature Review Using an Online Findings Archive</t>
+          <t>The stabilizing work of public actors. A study of the deployment of the Respect Module in French prisons</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01064-w</t>
+          <t>https://openalex.org/W7162820765</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -92,22 +92,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>health_mental_health</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Subjective Inequality and Well-being in South Korea: Generational Variations in the Mediating and Moderating Effects of Social Connectedness</t>
+          <t>The Role of Social Media Influencers in Promoting Therapeutic Compliance: Implications for Public Health Policy</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01072-w</t>
+          <t>https://openalex.org/W7137590217</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -117,7 +117,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>social, inequality, well-being</t>
+          <t>social</t>
         </is>
       </c>
     </row>
@@ -129,22 +129,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Emotional Closeness With Friends Is Associated With Sociodemographic Similarity and Personality Traits</t>
+          <t>Teachers’ involvement in the management of schools: example of France and French-speaking Belgium</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261465750?af=R</t>
+          <t>https://openalex.org/W7137708326</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>emotional, closeness</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -166,22 +166,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>governance_society</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rethinking social media metrics: Daily interaction valence and well‐being in university students</t>
+          <t>Is the university an enabling environment? A qualitative study examining the impact of university disability policy for staff</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>British Journal of Social Psychology</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70109?af=R</t>
+          <t>https://openalex.org/W7137577846</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -191,7 +191,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>social, well-being</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -208,17 +208,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Does perfectionism moderate the effects of gratitude on social connectedness and psychological distress?</t>
+          <t>Une étude a posteriori de la construction de l’intention entrepreneuriale chez les entrepreneurs agricoles d’Afrique subsaharienne</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The Journal of Positive Psychology</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/full/10.1080/17439760.2026.2697158?af=R</t>
+          <t>https://openalex.org/W7137759281</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -228,7 +228,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -245,17 +245,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>When Ballet Fails to Inspire Attraction: Trait Signals Override Occupational Cues in Mate Preferences</t>
+          <t>The Enlightenment of an Entrepreneur: A Multidisciplinary Exploration of Management, Psychology and Economic Theology</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261465751?af=R</t>
+          <t>https://openalex.org/W7137519157</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Publication Notice</t>
+          <t>Le projet design comme moyen de stimuler l’intention entrepreneuriale</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Current Directions in Psychological Science</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261454343?af=R</t>
+          <t>https://openalex.org/W7153402517</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -319,17 +319,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Introduction to the Special Issue on Human and Machine Intelligence</t>
+          <t>Intention entrepreneuriale : profils et vision stratégique. Étude de cas des étudiants algériens</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Current Directions in Psychological Science</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261450881?af=R</t>
+          <t>https://openalex.org/W7137767042</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -351,22 +351,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Does Testosterone Affect Cognitive Reflection? Evidence From a Double-Blind, Randomized Controlled Study of 1,000 Participants</t>
+          <t>Exploring the Entrepreneurial Intentions of Academic Inventors in an Emerging Context: The Case of Morocco</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Psychological Science</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261458325?af=R</t>
+          <t>https://openalex.org/W7137390646</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -376,7 +376,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>affect</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -388,22 +388,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Associations Between Arts Engagement and Well-Being, Happiness and Life Satisfaction in Hong Kong Adults: A Cross-Sectional, Household-Based Survey</t>
+          <t>Des villes en pixels aux cités réelles : influence des jeux vidéo sur l’architecture urbaine contemporaine</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01073-9</t>
+          <t>https://openalex.org/W7137693611</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -413,7 +413,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>well-being</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -430,17 +430,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A Thematic Co-Occurrence Analysis of Communal Coping Within and Between Surviving Parents and Emerging-Adult Children After Partner/Parental Death</t>
+          <t>Association Between Anxiety and RRBs in Autistic Youth: Role of Ethnicity</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>The Scholars Repository - LLU (Loma Linda University)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261465752?af=R</t>
+          <t>https://openalex.org/W7167182114</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -467,17 +467,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A Field Experiment Testing Whether Accountability Reduces Racial Gaps in Performance Evaluations</t>
+          <t>Transversalité pour la circularité et la sobriété à Grenoble</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Psychological Science</t>
+          <t>HAL (Le Centre pour la Communication Scientifique Directe)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261458988?af=R</t>
+          <t>https://doi.org/10.5281/zenodo.14763521</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -499,22 +499,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>education_learning</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Does Overconfidence Really Confer Adaptive Benefits to Children’s Learning?</t>
+          <t>Defying the Catholic Secondary School Enrollment Decline: A Case Study Exploring Strategic Enrollment Management Practices in an All-Boys Catholic High School</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Psychological Science</t>
+          <t>Seton Hall University eRepository (Seton Hall University)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261455283?af=R</t>
+          <t>https://openalex.org/W7160677245</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -536,22 +536,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The humanizing power of nostalgia: a pathway to psychological richness</t>
+          <t>Exploring the Relationships Between Emotional Intelligence, Perceived Organizational Support, Job Satisfaction, and Intent to Stay Among Minnesota School Nurses</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>The Journal of Positive Psychology</t>
+          <t>RED - a Repository of Digital Collections (Minnesota State University Moorhead)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/full/10.1080/17439760.2026.2697168?af=R</t>
+          <t>https://openalex.org/W7165284361</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>psychological richness</t>
+          <t>relationships, emotional</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Metacognitive and Interpersonal Intellectual Humility Are Asymmetrically Associated with Well-Being</t>
+          <t>Parasympathetic Activity and Inhibitory Control as Predictors of Health Behaviors</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Personality and Social Psychology Bulletin</t>
+          <t>CU Scholar (University of Colorado Boulder)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261457222?af=R</t>
+          <t>https://openalex.org/W7159747169</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>interpersonal, well-being</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -615,17 +615,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Imagine No Resources: Attention Is Selection and Normalization for Choice</t>
+          <t>児童・青年期の反応性愛着障害における腹側線条体の機能不全：機能的MRI 研究</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Perspectives on Psychological Science</t>
+          <t>Institutional Repositories DataBase (IRDB)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/17456916261446902?af=R</t>
+          <t>https://doi.org/10.34463/0002000763</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -647,22 +647,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Does Social Media Use Really Matter for Students’ Well-Being? The Cross-Cultural Generalizability Across 52 Societies</t>
+          <t>Pilot Evaluation Plan of Can-Do Maths</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>UCL Discovery (University College London)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01070-y</t>
+          <t>https://openalex.org/W7112920481</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>social, well-being</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -689,17 +689,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Bodies in and out of place: The racialized entanglements of occupying space</t>
+          <t>The Seven Noahide Laws</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>British Journal of Social Psychology</t>
+          <t>Seton Hall University eRepository (Seton Hall University)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70107?af=R</t>
+          <t>https://openalex.org/W7162613458</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -716,37 +716,37 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>reject</t>
+          <t>high</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Subjective Inequity Aversion: How Perceived Unfair Inequality Affects Subjective Well-being</t>
+          <t>The Ethical and Legal Complexities of Regulating Companion AI Chatbots</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Lund University Publications (Lund University)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01053-z</t>
+          <t>https://openalex.org/W7143585285</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t/>
+          <t>AI, chatbots</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>inequality, well-being</t>
+          <t>companion</t>
         </is>
       </c>
     </row>
@@ -763,17 +763,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Outgroup friendships and social influence in the development of adolescent attitudes toward secondary outgroups.</t>
+          <t>Setting Up Living Labs for Water Reuse in Water-Stressed Social-Hydrological Systems</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Journal of Personality and Social Psychology</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-90625-001</t>
+          <t>https://openalex.org/W7154662464</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -795,22 +795,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>education_learning</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Honour the Light in Every Soul: Awe Reduces Objectification via Self‐Transcendence</t>
+          <t>Refusing expectation? Class, masculinity and selfhood in a longitudinal analysis of young men’s educational transitions/ trajectories, age 10-22</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>European Journal of Social Psychology</t>
+          <t>UCL Discovery (University College London)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70095?af=R</t>
+          <t>https://openalex.org/W7125092985</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -837,17 +837,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Executive function and social behavior: Causal evidence from loading working memory and inhibitory control.</t>
+          <t>Motivations intrinsèque et extrinsèque comme déterminants de l’intention d’adoption des objets connectés en santé mobile</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: General</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-91214-001</t>
+          <t>https://openalex.org/W7154669314</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -869,22 +869,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>organization_work</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Configurational antecedents of employee green behavior: A mixed methods study.</t>
+          <t>Le rôle des influenceurs des médias sociaux dans la promotion de l’observance thérapeutique : enjeux et perspectives pour la santé publique</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: Applied</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-91431-001</t>
+          <t>https://openalex.org/W7137612268</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -906,22 +906,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Community as Medicine: A Qualitative Exploration of Meaningful Social Support and Health for Trans‐ and Gender‐Diverse People in England</t>
+          <t>Innovation et durabilité : la cyclologistique comme vecteur de transformation de la logistique hospitalière</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>European Journal of Social Psychology</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70093?af=R</t>
+          <t>https://openalex.org/W7154662957</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>social, social support, gender</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -943,22 +943,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>mind_acceptance</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Children’s Third-Party Punishment Reveals a Genuine Concern for Fairness and Justice</t>
+          <t>Innovation amidst Turmoil, Part 2: Narratives and Sensemaking among German Managers during the Pandemic</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Perspectives on Psychological Science</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/17456916261454645?af=R</t>
+          <t>https://openalex.org/W7162719679</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -985,17 +985,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Chaos Theory and Child Development: Quantifying Nonlinear Pathways of Growth</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Perspectives on Psychological Science</t>
+          <t>RUCforsk (Roskilde University)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/17456916261451880?af=R</t>
+          <t>https://openalex.org/W7165701504</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1017,22 +1017,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Supporting in Ways That Do Not Align With What We Feel, Believe, or Want: Theorizing About Deceptive/Reluctant Support Provision in Interpersonal Relationships</t>
+          <t>Diasporic Sikh masculinities in Ranj Dhaliwal’s "Daaku" and Gautam Malkani’s "Londonstani"</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>cIRcle (University of British Columbia)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463317?af=R</t>
+          <t>https://doi.org/10.14288/1.0105084</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>relationships, interpersonal</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1054,22 +1054,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Linking Attachment Orientations and Romantic Relationship Quality: The Role of Trait Mindfulness and Relationship Mindfulness</t>
+          <t>Business Model Innovation among Startups and Its Future Research Trends: A Systematic Review and Bibliometric Analysis of Relevant Literature</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463850?af=R</t>
+          <t>https://openalex.org/W7137489039</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1079,14 +1079,14 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>relationship, attachment</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>reject</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1096,22 +1096,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>How Awe in Nonwork Activities Promotes Proactive Behavior in Employees: A Spillover Model</t>
+          <t>Anticiper et écrire la place des robots dans l’industrie du futur : une approche science-fictionnelle et métaphorique</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Cairn.info</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01074-8</t>
+          <t>https://openalex.org/W7164448054</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t/>
+          <t>robots</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1128,22 +1128,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>consumer_marketing</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Globalize the Intifada: Integrating Historical Materialism to Critically Examine Pro‐Palestine Solidarity Motivations in the ‘I'm Not Palestinian but’ Action</t>
+          <t>From Embedded Finance to Embedded Obligation: A Law-and-Economics Theory of Consumer Protection in Platform-Mediated Financial Services</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>European Journal of Social Psychology</t>
+          <t>Open MIND</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70092?af=R</t>
+          <t>https://doi.org/10.17613/sb76m-v2e23</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1165,22 +1165,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>mind_acceptance</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>How Does the Mind Grow? Cross-Cultural Intuitive Theories of Mental Development</t>
+          <t>Natural Agents, Complex Systems and Uncertain Environments: Results from Simulations on Heuristic Organizations</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Psychological Science</t>
+          <t>HAL (Le Centre pour la Communication Scientifique Directe)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261453926?af=R</t>
+          <t>https://openalex.org/W7134097949</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1202,22 +1202,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>organization_work</t>
+          <t>consumer_marketing</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Enacting a Eudaimonic View: Development and Validation of a Questionnaire for Eudaimonic Well-Being in the Workplace</t>
+          <t>Smart service experience and consumer loyalty in Saudi Arabian smart hotels: The mediating roles of tourist happiness and value co-creation</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Digital Commons - University of South Florida (University of South Florida)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01048-w</t>
+          <t>https://doi.org/10.5038/2640-6489.11.2.1385</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>well-being</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1244,17 +1244,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Perception and action as one: Re-integrating research on human action through event files.</t>
+          <t>Reconstruction and Renaissance of Dongbei China:A Multimodal Metaphor Analysis of New Media on Harbin</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Psychological Review</t>
+          <t>Research Explorer (The University of Manchester)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-89081-001</t>
+          <t>https://openalex.org/W7130910808</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1276,22 +1276,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Conveying (discrete) emotionality with novel words.</t>
+          <t>Place label nudges : How place attachment shapes recycling choice</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: General</t>
+          <t>Lancaster EPrints (Lancaster University)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-89054-001</t>
+          <t>https://openalex.org/W7164714552</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t/>
+          <t>attachment</t>
         </is>
       </c>
     </row>
@@ -1313,22 +1313,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>mind_acceptance</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Associations Between Self-Acceptance, Cognitive Reappraisal, and Life Satisfaction among Adolescents: A Three-Wave Study</t>
+          <t>Relationship of COVID-19-Related Racial Discrimination and Oppressed Identities on Chinese American Mental Health</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>USF Scholarship Repository (University of San Francisco)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01071-x</t>
+          <t>https://openalex.org/W7164619148</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t/>
+          <t>relationship, mental health</t>
         </is>
       </c>
     </row>
@@ -1350,22 +1350,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>governance_society</t>
+          <t>health_mental_health</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>When and Why Beliefs About the Causes of a Policy Problem Predict Policy Support</t>
+          <t>Investigating the Role of Patient-Provider Interaction Quality and Illness Interference in Patients' Basic Psychological Need Fulfillment and Subjective Well-Being</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Personality and Social Psychology Bulletin</t>
+          <t>Digital Commons - USU (Utah State University)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261456781?af=R</t>
+          <t>https://openalex.org/W7163462893</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t/>
+          <t>well-being</t>
         </is>
       </c>
     </row>
@@ -1387,22 +1387,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Transforming the Youth Mental Health Workforce</t>
+          <t>Historical Inquiry-Based Lessons in World History Classrooms: Creating Opportunities for Historical Thinking</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Current Directions in Psychological Science</t>
+          <t>Digital Commons - USU (Utah State University)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261436736?af=R</t>
+          <t>https://openalex.org/W7169636114</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>mental health</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1424,22 +1424,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>education_learning</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Sexuality as Gendered: Understanding the Intertwining of Sexual Orientation and Gender Across Individual and Sociocultural Domains</t>
+          <t>Evolving Roles: School Counselors Addressing Mental Health in PK-12 Education</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Current Directions in Psychological Science</t>
+          <t>Digital Commons - USU (Utah State University)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261438050?af=R</t>
+          <t>https://openalex.org/W7169634416</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>mental health</t>
         </is>
       </c>
     </row>
@@ -1461,22 +1461,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mix and Match: Frequency of Public Affection Sharing as a Predictor of Well-being in White versus Interracial Relationships</t>
+          <t>A Qualitative Study of Immigration Trauma, Posttraumatic Growth, and the College Experience Among MENA Immigrant Students</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>Digital Commons at National Lewis University (National Lewis University)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463580?af=R</t>
+          <t>https://openalex.org/W7159904425</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1486,14 +1486,14 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>relationships, well-being</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>reject</t>
+          <t>high</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1503,27 +1503,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Intergroup Contact and Belonging Among Ethiopian Jews in Ethiopia</t>
+          <t>Towards Scalable and Ecological Methods for Early Social Development Research: Validating Automated Facial Expression Estimation in Egocentric Video</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Personality and Social Psychology Bulletin</t>
+          <t>White Rose Research Online (University of Leeds, The University of Sheffield, University of York)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261454081?af=R</t>
+          <t>https://openalex.org/W7161364511</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t/>
+          <t>automated</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>belonging</t>
+          <t>social</t>
         </is>
       </c>
     </row>
@@ -1535,22 +1535,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Developmental Change in Cortisol Reactivity Following Early Deprivation: Potential Links to Emotional Adjustment</t>
+          <t>Does Self-Projection Have a Dominant Temporal Direction? In Nine Countries, People Feel More Similar to Their Future Than Past Selves</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Current Directions in Psychological Science</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261439665?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261467790?af=R</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1572,22 +1572,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>A Taxonomy of Data Synthesis</t>
+          <t>The influence of college students’ “Wan Geng” motivation on emotion regulation self-efficacy</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Personality and Social Psychology Bulletin</t>
+          <t>Frontiers in Psychology</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261451901?af=R</t>
+          <t>https://doi.org/10.3389/fpsyg.2026.1802652</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t/>
+          <t>emotion</t>
         </is>
       </c>
     </row>
@@ -1609,22 +1609,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>consumer_marketing</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>A Meta‐Analysis of Self–Other Differences in Prejudice</t>
+          <t>The Political Economy of Embedded Marketing in the Television Quiz Show Family 100: A Qualitative Study</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>European Journal of Social Psychology</t>
+          <t>Glosains Jurnal Sains Global Indonesia</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70094?af=R</t>
+          <t>https://doi.org/10.59784/glosains.v7i3.795</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1646,22 +1646,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>A Cross-National Comparison of Ghosting Knowledge, Attitudes, Intentions, and Behaviors in Friendships and Romantic Relationships Spanning Twelve Countries</t>
+          <t>Social Media is Shifting the Values in Our Societies: An Increase in People’s Achievement and Conformity Orientation</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463579?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261461314?af=R</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>relationships</t>
+          <t>social</t>
         </is>
       </c>
     </row>
@@ -1683,22 +1683,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Romantic Relationships and Socioeconomic Status as Independent Predictors of Health and Wellbeing: Evidence From the United States and Spain</t>
+          <t>Rethink beauty, change how you feel: Mediating role of effort invested</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>Acta Psychologica</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463571?af=R</t>
+          <t>https://doi.org/10.1016/j.actpsy.2026.107459</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>relationships, wellbeing</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1725,17 +1725,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Prospects of Downward Mobility Cause Status Anxiety and Life Dissatisfaction</t>
+          <t>On the role of verbal semantics in question embedding: the case of to know</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Personality and Social Psychology Bulletin</t>
+          <t>Linguistics and Philosophy</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261451296?af=R</t>
+          <t>https://doi.org/10.1007/s10988-026-09464-0</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -1752,37 +1752,37 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>reject</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>On the Inner Workings of the Person–Culture Match Effect on Well-Being</t>
+          <t>Machiavellianism, Bullying, and Manipulation Fears in the AI Work Environment</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Social Psychological and Personality Science</t>
+          <t>Journal of Leadership Accountability and Ethics</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/19485506261453640?af=R</t>
+          <t>https://doi.org/10.33423/m996x860</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t/>
+          <t>AI</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>well-being</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1794,22 +1794,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Not All Practice Is Created Equal: Longitudinal Evidence From Over 40,000 Chess Players</t>
+          <t>Family Dynamics And Pro-Social Competence Of College Students In Osun State, Nigeria</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Psychological Science</t>
+          <t>F1000Research</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261452568?af=R</t>
+          <t>https://doi.org/10.12688/f1000research.183020.1</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -1819,44 +1819,44 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>equal</t>
+          <t>social</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>reject</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>The impact of “relational” Artificial Intelligence on human well-being: A self-determination theory analysis.</t>
+          <t>Analytical Study on Unsolved Question and Mysteries of the Universe and Wisdom from Holly Book</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Journal of Personality and Social Psychology</t>
+          <t>Transactions on Engineering and Computing Sciences</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-87670-001</t>
+          <t>https://doi.org/10.14738/tecs.1404.11991</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>artificial intelligence</t>
+          <t/>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>relational, well-being</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1873,17 +1873,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Cumulative adverse childhood experiences and parent-reported allergic conditions and asthma among U.S. children: A nationally representative study.</t>
+          <t>Moved by the Lightest Touch of Meaning: Even Minimal Significance Matters for Motivation From Childhood</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>American Psychologist</t>
+          <t>Psychological Science</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-88271-001</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261462874?af=R</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -1905,22 +1905,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>education_learning</t>
+          <t>organization_work</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Associative learning explains “intuitive statistics” in animals.</t>
+          <t>Does losing your job change your personality? Findings from a 16-year longitudinal study of Mexican-origin adults.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Psychological Review</t>
+          <t>Journal of Personality and Social Psychology</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-87718-001</t>
+          <t>https://psycnet.apa.org/record/2027-98633-001</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -1942,22 +1942,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>A reciprocal model of practice and skill: Navigating between dropout and expertise.</t>
+          <t>Do money and time change who you are? A continuous time meta-analysis and review of reciprocal relationships between personality traits and income.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Psychological Review</t>
+          <t>Psychological Bulletin</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-87672-001</t>
+          <t>https://psycnet.apa.org/record/2027-99625-001</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t/>
+          <t>relationships</t>
         </is>
       </c>
     </row>
@@ -1979,22 +1979,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Why Did the Gender Gap in Adolescent Life Satisfaction Grow? Evaluating Methodological and Demographic Explanations</t>
+          <t>Stable Worldviews or Context-Sensitive Systems? Longitudinal Evidence on the Development of Epistemically Suspect Beliefs Across Two Sociopolitical Contexts</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01068-6</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261463908?af=R</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -2021,17 +2021,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Eudaimonic but not Hedonic or Extrinsic Motives Predict Less Academic Distress Among Adolescents—Indirect Effect via Flourishing</t>
+          <t>Replication of “Procrastination, Deadlines, and Performance: Self-Control by Precommitment”</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Psychological Science</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01069-5</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261460772?af=R</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2053,22 +2053,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Correction: Development of a Holistic Mental Health Item Bank for Use in the General Population</t>
+          <t>To Regulate or Not to Regulate? Situational and Individual Differences in Emotion Regulation Initiation in Daily Life</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01065-9</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261461318?af=R</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>mental health</t>
+          <t>emotion</t>
         </is>
       </c>
     </row>
@@ -2095,17 +2095,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The role of moral identity in ideological obsession and violent extremism</t>
+          <t>The role of children’s media in White, U.S. children’s developing racial biases.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>British Journal of Social Psychology</t>
+          <t>American Psychologist</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70106?af=R</t>
+          <t>https://psycnet.apa.org/record/2027-94892-001</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2132,17 +2132,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Physical actions shape moral choices: Environment-directed movements reduce cheating in young children.</t>
+          <t>Perceived Pain Sensitivity and Treatment Recommendations for Socially Mobile Individuals: The Mediating Role of Perceived Tenacity</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: General</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-86918-001</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261464676?af=R</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t/>
+          <t>socially</t>
         </is>
       </c>
     </row>
@@ -2169,17 +2169,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Correction to ‘Digitizing fear: Identity, threat and collective mobilization through social media posts during the 2021 election campaigns in West Bengal, India’</t>
+          <t>Lonnie R. Snowden (1947–2025).</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>British Journal of Social Psychology</t>
+          <t>American Psychologist</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70108?af=R</t>
+          <t>https://psycnet.apa.org/record/2027-96114-001</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -2201,22 +2201,22 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>governance_society</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Global mapping of happiness: mechanisms, drivers, and pathways to societal happiness</t>
+          <t>A two-dimensional framework for prior knowledge in goal-directed navigation.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>The Journal of Positive Psychology</t>
+          <t>Journal of Experimental Psychology: General</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/full/10.1080/17439760.2026.2684517?af=R</t>
+          <t>https://psycnet.apa.org/record/2027-97795-001</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2233,37 +2233,37 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>reject</t>
+          <t>high</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Eye Glint as a Novel Perceptual Cue in Human Vision</t>
+          <t>AI-Generated Empathy: Opportunities, Limits, and Future Directions</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Psychological Science</t>
+          <t>Current Directions in Psychological Science</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261446892?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261444274?af=R</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t/>
+          <t>AI, AI-generated</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t/>
+          <t>empathy</t>
         </is>
       </c>
     </row>
@@ -2275,22 +2275,22 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>organization_work</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Towards a theory of fostering workplace dignity across social identity differences: Practices of exemplary supervisors</t>
+          <t>Older Sibling Prosocial Behavior Toward Younger Siblings During Adolescence: A Multi-Informant Multi-Method Investigation</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>The Journal of Positive Psychology</t>
+          <t>Journal of Social and Personal Relationships</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/full/10.1080/17439760.2026.2684660?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261469656?af=R</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -2312,12 +2312,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The Friends They Have and the Friends They Want: Why Friendship Aspirations Usually Fail</t>
+          <t>Bystander Reactions to Economic Abuse: The Role of Moral Evaluation and Victim Blaming</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261461795?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261467470?af=R</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2337,14 +2337,14 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>friendship</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>reject</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2354,22 +2354,22 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Combining Psychology With Artificial Intelligence: What Could Possibly Go Wrong?</t>
+          <t>Unconscious mental content in implicit evaluation: Evidence from misprediction.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Current Directions in Psychological Science</t>
+          <t>Journal of Personality and Social Psychology</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261438379?af=R</t>
+          <t>https://psycnet.apa.org/record/2027-94884-001</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>artificial intelligence</t>
+          <t/>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2391,17 +2391,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The relative psychometric function: A general analysis framework for relating psychological processes.</t>
+          <t>Tightening up under threat: Social class shapes the strength of norms.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Psychological Review</t>
+          <t>Journal of Personality and Social Psychology</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-83723-001</t>
+          <t>https://psycnet.apa.org/record/2027-95666-001</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t/>
+          <t>social</t>
         </is>
       </c>
     </row>
@@ -2423,22 +2423,22 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>health_mental_health</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Power to Care for Oneself: Power Increases Self‐Compassion</t>
+          <t>The Benefits of Prosocial Behavior for Mental and Physical Health: A Neuroscience Approach</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>European Journal of Social Psychology</t>
+          <t>Current Directions in Psychological Science</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70090?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261459027?af=R</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2465,17 +2465,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Revisiting Social Anhedonia: Beyond Monolithic Assessments and Interventions</t>
+          <t>Internalized racism as a self-regulatory system: The internalized racism process model.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Current Directions in Psychological Science</t>
+          <t>Psychological Review</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261436743?af=R</t>
+          <t>https://psycnet.apa.org/record/2027-94888-001</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -2497,22 +2497,22 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Reducing Intergroup Bias Towards Stigmatised Groups: How Intersectionality Models Advance Beyond Traditional Models of Social Categorisation</t>
+          <t>Internal domain generality for ensemble perception of average orientation: Comparing and integrating information from multiple stimulus categories.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>European Journal of Social Psychology</t>
+          <t>Journal of Experimental Psychology: General</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70091?af=R</t>
+          <t>https://psycnet.apa.org/record/2027-94891-001</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -2539,17 +2539,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Practice guidelines regarding psychologists’ involvement in pharmacological issues.</t>
+          <t>Beyond synchrony: Why disengagement can sometimes be the healthiest choice.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>American Psychologist</t>
+          <t>Psychological Review</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-83950-001</t>
+          <t>https://psycnet.apa.org/record/2027-94894-001</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -2576,17 +2576,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Natural disaster, social cohesion, and prosociality: A natural experiment.</t>
+          <t>Beyond WEIRD Humans and STRANGE Dogs: Using Big-Team Science to Improve Generalizability and Reproducibility in Comparative Psychology</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>American Psychologist</t>
+          <t>Current Directions in Psychological Science</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-83810-001</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261450055?af=R</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -2608,22 +2608,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Listening across the divide: High-quality listening promotes speakers’ state well-being through basic psychological need satisfaction during disagreements.</t>
+          <t>Experimental tests of the tertiary transfer effect of intergroup contact: Addressing valence, prototypicality and moderators</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Journal of Personality and Social Psychology</t>
+          <t>British Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-84452-001</t>
+          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70113?af=R</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>well-being</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -2645,22 +2645,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>gender_equality</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Is my loneliness killing me? Effects of loneliness and social isolation on transitions between cognitive status categories and death.</t>
+          <t>As warm as competent, really? On the importance of stereotype facets in the context of autism</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Journal of Personality and Social Psychology</t>
+          <t>British Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-84465-001</t>
+          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70112?af=R</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>social, loneliness</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -2687,17 +2687,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Intuitive Judgments of Strangers Are More Popular but Not More Accurate Than Deliberate Ones</t>
+          <t>No Evidence for Self-Esteem Effects on Aggression: Findings From a Multi-Year, Multi-Informant Longitudinal Study of Mexican-Origin Families</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Social Psychological and Personality Science</t>
+          <t>Psychological Science</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/19485506261452705?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261459011?af=R</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -2724,17 +2724,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>How autobiographical memory serves morality: Prevalence and properties of memories with moral content.</t>
+          <t>Dominance meets competence: A socio‐ecological perspective on leadership and human social hierarchies</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: General</t>
+          <t>British Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-83836-001</t>
+          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70111?af=R</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t/>
+          <t>social</t>
         </is>
       </c>
     </row>
@@ -2756,22 +2756,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>education_learning</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>From chunks to schemas: Learning in the Hebb repetition paradigm.</t>
+          <t>Why the Big Five personality traits are composites, not common causes: Implications for measurement, prediction, and causal inference.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: General</t>
+          <t>Psychological Review</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-83839-001</t>
+          <t>https://psycnet.apa.org/record/2027-91833-001</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -2798,17 +2798,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Formal Modeling as Theoretical Glue between Laboratory and Naturalistic Studies of Memory</t>
+          <t>Universal pluralism: Appreciating and exploring both similarity and difference across people and cultures.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Perspectives on Psychological Science</t>
+          <t>American Psychologist</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/17456916261419428?af=R</t>
+          <t>https://psycnet.apa.org/record/2027-92049-001</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -2835,17 +2835,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>What It Means to Put Children First: A Mixed-Method Investigation of Child-Centric Parenting</t>
+          <t>Populism and the Pandemic: How the Covid‐Sceptic Movement Mobilised Opposition to Covid Measures</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>European Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261459484?af=R</t>
+          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70097?af=R</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -2867,22 +2867,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Meaning in life, basic psychological needs, and subjective well-being: A Meta-Analytic Structural Equation Modeling Approach</t>
+          <t>On the Goals and Limitations of Psychological Science: Some Thoughts in Memory of Daniel Kahneman</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>The Journal of Positive Psychology</t>
+          <t>Perspectives on Psychological Science</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/full/10.1080/17439760.2026.2683403?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/17456916261417988?af=R</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -2892,7 +2892,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>well-being, meaning in life</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -2909,17 +2909,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Excellence in media: the effects of ability-based awe videos on prosocial intention and self-improvement</t>
+          <t>Does the variance of personality traits change across the lifespan? A meta-analytic review of longitudinal studies.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>The Journal of Positive Psychology</t>
+          <t>Psychological Bulletin</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/full/10.1080/17439760.2026.2683406?af=R</t>
+          <t>https://psycnet.apa.org/record/2027-92059-001</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -2941,22 +2941,22 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Who Fancies Whom? Investigating Adolescent Romantic Interests</t>
+          <t>Did politically engaged individuals construe the COVID‐19 pandemic primarily as a security threat, a welfare threat, or both? Understanding differential emotional and ideological responses to threats through the lens of THEISM</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>British Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261460936?af=R</t>
+          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70101?af=R</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t/>
+          <t>emotional</t>
         </is>
       </c>
     </row>
@@ -2983,17 +2983,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>The effects of counterfactual thinking on unilateral forgiveness: Can victims do it on their own?</t>
+          <t>Boosting Media Literacy Using Lateral Reading and Online Search Interventions</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: Applied</t>
+          <t>Psychological Science</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-82653-001</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261453813?af=R</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Racial Oppression, Self-Efficacy, and Avoidance of Interpersonal Intimacy Among Queer Men of Color: A Longitudinal Investigation</t>
+          <t>Emotional Closeness With Friends Is Associated With Sociodemographic Similarity and Personality Traits</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261460502?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261465750?af=R</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3040,7 +3040,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>interpersonal, intimacy</t>
+          <t>emotional, closeness</t>
         </is>
       </c>
     </row>
@@ -3057,17 +3057,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Nostalgia Increases Psychological Richness in Life</t>
+          <t>Rethinking social media metrics: Daily interaction valence and well‐being in university students</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Social Psychological and Personality Science</t>
+          <t>British Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/19485506261454720?af=R</t>
+          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70109?af=R</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>psychological richness</t>
+          <t>social, well-being</t>
         </is>
       </c>
     </row>
@@ -3089,22 +3089,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Morality cut both ways: The role of cognition and emotion in attitude moralization and demoralization.</t>
+          <t>When Ballet Fails to Inspire Attraction: Trait Signals Override Occupational Cues in Mate Preferences</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Journal of Personality and Social Psychology</t>
+          <t>Journal of Social and Personal Relationships</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-82786-001</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261465751?af=R</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>emotion</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -3126,22 +3126,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Maternal Stress and Bonding in the COVID-19 Pandemic: Mothers’ Relationship Quality With the Partner as a Resilience Factor</t>
+          <t>Publication Notice</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>Current Directions in Psychological Science</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261459477?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261454343?af=R</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>relationship</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -3163,22 +3163,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Dyadic Effects of Relationship Dissatisfaction and Impulsivity on Physical and Psychological Intimate Partner Violence Perpetration</t>
+          <t>Introduction to the Special Issue on Human and Machine Intelligence</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>Current Directions in Psychological Science</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261455928?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261450881?af=R</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>relationship, intimate</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -3200,22 +3200,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>‘Far right just means anyone who wants to support British values’: Mobilizing ‘British values’ talk in discussions of the August 2024 UK race riots</t>
+          <t>Does Testosterone Affect Cognitive Reflection? Evidence From a Double-Blind, Randomized Controlled Study of 1,000 Participants</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>British Journal of Social Psychology</t>
+          <t>Psychological Science</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70093?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261458325?af=R</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t/>
+          <t>affect</t>
         </is>
       </c>
     </row>
@@ -3242,17 +3242,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Are Free Will Believers Happier? Converging Evidence From Daily Life and Experimental Research</t>
+          <t>A Thematic Co-Occurrence Analysis of Communal Coping Within and Between Surviving Parents and Emerging-Adult Children After Partner/Parental Death</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Social Psychological and Personality Science</t>
+          <t>Journal of Social and Personal Relationships</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/19485506261450242?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261465752?af=R</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3279,17 +3279,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>A Theoretical Framework and The Development of a Multidimensional Scale of Purpose in Life</t>
+          <t>A Field Experiment Testing Whether Accountability Reduces Racial Gaps in Performance Evaluations</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Journal of Happiness Studies</t>
+          <t>Psychological Science</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s10902-026-01067-7</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261458988?af=R</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3311,22 +3311,22 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>education_learning</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>From Family to Partnership: Intrusive Parenting and Couple Identity Through Dyadic Coping</t>
+          <t>Does Overconfidence Really Confer Adaptive Benefits to Children’s Learning?</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Journal of Social and Personal Relationships</t>
+          <t>Psychological Science</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261459147?af=R</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261455283?af=R</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3348,22 +3348,22 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>health_mental_health</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>The predictive validity of vocational interests for life outcomes across adulthood.</t>
+          <t>Metacognitive and Interpersonal Intellectual Humility Are Asymmetrically Associated with Well-Being</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Journal of Personality and Social Psychology</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-80205-001</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261457222?af=R</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t/>
+          <t>interpersonal, well-being</t>
         </is>
       </c>
     </row>
@@ -3385,22 +3385,22 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Interventions to reduce implicit weight bias: A focus on mechanisms and individual differences.</t>
+          <t>Imagine No Resources: Attention Is Selection and Normalization for Choice</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: General</t>
+          <t>Perspectives on Psychological Science</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-80206-001</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/17456916261446902?af=R</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3427,17 +3427,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>International Competences for Undergraduate Psychology (ICUP) : A constructive shift for psychology?</t>
+          <t>Bodies in and out of place: The racialized entanglements of occupying space</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>American Psychologist</t>
+          <t>British Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-79792-001</t>
+          <t>https://bpspsychub.onlinelibrary.wiley.com/doi/10.1111/bjso.70107?af=R</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -3459,22 +3459,22 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Bridging Bayesian and representational theories of memory to predict memory bias.</t>
+          <t>Outgroup friendships and social influence in the development of adolescent attitudes toward secondary outgroups.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: General</t>
+          <t>Journal of Personality and Social Psychology</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-79787-001</t>
+          <t>https://psycnet.apa.org/record/2027-90625-001</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -3484,14 +3484,14 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t/>
+          <t>social</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>reject</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -3501,22 +3501,22 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Artificial intelligence and machines are capable of harm, but not of experiencing punishment.</t>
+          <t>Honour the Light in Every Soul: Awe Reduces Objectification via Self‐Transcendence</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Journal of Experimental Psychology: General</t>
+          <t>European Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-80422-001</t>
+          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70095?af=R</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>artificial intelligence</t>
+          <t/>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -3538,17 +3538,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>A taxonomy of discriminatory behavior.</t>
+          <t>Executive function and social behavior: Causal evidence from loading working memory and inhibitory control.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Psychological Review</t>
+          <t>Journal of Experimental Psychology: General</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://psycnet.apa.org/record/2027-80429-001</t>
+          <t>https://psycnet.apa.org/record/2027-91214-001</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t/>
+          <t>social</t>
         </is>
       </c>
     </row>
@@ -3570,22 +3570,22 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>organization_work</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>“Friend or foe?” the ironic effect of speaking the minority's language in intergroup conflicts: Palestinian reactions to Jewish-Israelis using Arabic</t>
+          <t>Configurational antecedents of employee green behavior: A mixed methods study.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Journal of Experimental Psychology: Applied</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000739?dgcid=rss_sd_all</t>
+          <t>https://psycnet.apa.org/record/2027-91431-001</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>friend</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -3607,22 +3607,22 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Why do people dislike gender role violators? A test of three models</t>
+          <t>Community as Medicine: A Qualitative Exploration of Meaningful Social Support and Health for Trans‐ and Gender‐Diverse People in England</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>European Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000569?dgcid=rss_sd_all</t>
+          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70093?af=R</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>social, social support, gender</t>
         </is>
       </c>
     </row>
@@ -3644,22 +3644,22 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>governance_society</t>
+          <t>mind_acceptance</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>When society feels broken: How perceptions of anomie shape donation tendencies across cultures</t>
+          <t>Children’s Third-Party Punishment Reveals a Genuine Concern for Fairness and Justice</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Perspectives on Psychological Science</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S002210312600051X?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/17456916261454645?af=R</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -3686,17 +3686,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>When rightness is wrong: Chronic prevention orientation predicts cardiovascular threat responses under regulatory fit</t>
+          <t>Chaos Theory and Child Development: Quantifying Nonlinear Pathways of Growth</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Perspectives on Psychological Science</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000508?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/17456916261451880?af=R</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -3718,22 +3718,22 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>We are nature: Engaging with community and nature to promote well-being and address environmental challenges</t>
+          <t>Supporting in Ways That Do Not Align With What We Feel, Believe, or Want: Theorizing About Deceptive/Reluctant Support Provision in Interpersonal Relationships</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Journal of Social and Personal Relationships</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X2600062X?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463317?af=R</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>well-being</t>
+          <t>relationships, interpersonal</t>
         </is>
       </c>
     </row>
@@ -3755,22 +3755,22 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Using intersectional implicit association measures does not consistently improve the predictive validity of the implicit association test</t>
+          <t>Linking Attachment Orientations and Romantic Relationship Quality: The Role of Trait Mindfulness and Relationship Mindfulness</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Journal of Social and Personal Relationships</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000491?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463850?af=R</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t/>
+          <t>relationship, attachment</t>
         </is>
       </c>
     </row>
@@ -3797,17 +3797,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Unequal participation: How low socioeconomic status hinders political engagement</t>
+          <t>Globalize the Intifada: Integrating Historical Materialism to Critically Examine Pro‐Palestine Solidarity Motivations in the ‘I'm Not Palestinian but’ Action</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>European Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000521?dgcid=rss_sd_all</t>
+          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70092?af=R</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -3829,22 +3829,22 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>mind_acceptance</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Two wrongs is what makes it more right: How retaliatory incivility receives social leniency</t>
+          <t>How Does the Mind Grow? Cross-Cultural Intuitive Theories of Mental Development</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Psychological Science</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000430?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261453926?af=R</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -3866,22 +3866,22 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Trust under watch: Relational models and the context-dependent nature of monitoring</t>
+          <t>Perception and action as one: Re-integrating research on human action through event files.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Psychological Review</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S002210312600065X?dgcid=rss_sd_all</t>
+          <t>https://psycnet.apa.org/record/2027-89081-001</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>relational</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -3903,22 +3903,22 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>education_learning</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Tracking connections, not content: How working memory shapes content and social learning in online networks</t>
+          <t>Conveying (discrete) emotionality with novel words.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Journal of Experimental Psychology: General</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000557?dgcid=rss_sd_all</t>
+          <t>https://psycnet.apa.org/record/2027-89054-001</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -3940,22 +3940,22 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>governance_society</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>The spread of fear: Perceptual deindividuation drives racial bias in threat generalization</t>
+          <t>When and Why Beliefs About the Causes of a Policy Problem Predict Policy Support</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000648?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261456781?af=R</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -3977,22 +3977,22 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>health_mental_health</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>The new identitarians: How the behavioral movement and psychology in general have been ideologically captured</t>
+          <t>Transforming the Youth Mental Health Workforce</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Current Directions in Psychological Science</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000643?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261436736?af=R</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -4002,7 +4002,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t/>
+          <t>mental health</t>
         </is>
       </c>
     </row>
@@ -4014,22 +4014,22 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>gender_equality</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>The effects of anonymity in volunteer's dilemmas</t>
+          <t>Sexuality as Gendered: Understanding the Intertwining of Sexual Orientation and Gender Across Individual and Sociocultural Domains</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Directions in Psychological Science</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000594?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261438050?af=R</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t/>
+          <t>gender</t>
         </is>
       </c>
     </row>
@@ -4051,22 +4051,22 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>organization_work</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>The effect of frameswitching on perceptions of decisiveness, creativity, and job fit</t>
+          <t>Mix and Match: Frequency of Public Affection Sharing as a Predictor of Well-being in White versus Interracial Relationships</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Journal of Social and Personal Relationships</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000429?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463580?af=R</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t/>
+          <t>relationships, well-being</t>
         </is>
       </c>
     </row>
@@ -4093,17 +4093,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>The Decolonization of Museums</t>
+          <t>Intergroup Contact and Belonging Among Ethiopian Jews in Ethiopia</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000680?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261454081?af=R</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t/>
+          <t>belonging</t>
         </is>
       </c>
     </row>
@@ -4125,22 +4125,22 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Testing the psychological distinctiveness of proscriptive and prescriptive moral norms: A replication and extension of Janoff-Bulman et al. (2009)</t>
+          <t>Developmental Change in Cortisol Reactivity Following Early Deprivation: Potential Links to Emotional Adjustment</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Directions in Psychological Science</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000776?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09637214261439665?af=R</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -4150,7 +4150,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t/>
+          <t>emotional</t>
         </is>
       </c>
     </row>
@@ -4167,17 +4167,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Strategically prosocial: Using acts of kindness to secure more valuable interaction partners</t>
+          <t>A Taxonomy of Data Synthesis</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000697?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261451901?af=R</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -4204,17 +4204,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Selective ignorance? The role of the information target in allocation decisions</t>
+          <t>A Meta‐Analysis of Self–Other Differences in Prejudice</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>European Journal of Social Psychology</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000892?dgcid=rss_sd_all</t>
+          <t>https://onlinelibrary.wiley.com/doi/10.1002/ejsp.70094?af=R</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -4236,22 +4236,22 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Research on microaggressions and their impact assesses neither microaggressions nor their impact</t>
+          <t>A Cross-National Comparison of Ghosting Knowledge, Attitudes, Intentions, and Behaviors in Friendships and Romantic Relationships Spanning Twelve Countries</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Journal of Social and Personal Relationships</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000631?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463579?af=R</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t/>
+          <t>relationships</t>
         </is>
       </c>
     </row>
@@ -4273,22 +4273,22 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Rational and irrational sociopolitical anxiety: Fear of cancellation</t>
+          <t>Romantic Relationships and Socioeconomic Status as Independent Predictors of Health and Wellbeing: Evidence From the United States and Spain</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Journal of Social and Personal Relationships</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000710?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/02654075261463571?af=R</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t/>
+          <t>relationships, wellbeing</t>
         </is>
       </c>
     </row>
@@ -4315,17 +4315,17 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Racism in the science and practice of psychotherapy</t>
+          <t>Prospects of Downward Mobility Cause Status Anxiety and Life Dissatisfaction</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Personality and Social Psychology Bulletin</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000722?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/01461672261451296?af=R</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -4347,22 +4347,22 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>health_mental_health</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Psychotherapy populations that are overlooked due to sociopolitical bias</t>
+          <t>On the Inner Workings of the Person–Culture Match Effect on Well-Being</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Social Psychological and Personality Science</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000692?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/19485506261453640?af=R</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t/>
+          <t>well-being</t>
         </is>
       </c>
     </row>
@@ -4384,22 +4384,22 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>governance_society</t>
+          <t>gender_equality</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Politicizing CBT: Reflections on the boundaries between therapy and society</t>
+          <t>Not All Practice Is Created Equal: Longitudinal Evidence From Over 40,000 Chess Players</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Psychological Science</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000837?dgcid=rss_sd_all</t>
+          <t>https://journals.sagepub.com/doi/abs/10.1177/09567976261452568?af=R</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -4409,44 +4409,44 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t/>
+          <t>equal</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>reject</t>
+          <t>high</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Playing it safe: Negotiators avoid uncertainty and reach safer, but less integrative agreements</t>
+          <t>The impact of “relational” Artificial Intelligence on human well-being: A self-determination theory analysis.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Journal of Personality and Social Psychology</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000545?dgcid=rss_sd_all</t>
+          <t>https://psycnet.apa.org/record/2027-87670-001</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t/>
+          <t>artificial intelligence</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t/>
+          <t>relational, well-being</t>
         </is>
       </c>
     </row>
@@ -4463,17 +4463,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Persuasion via intermediaries: The pull of extremity</t>
+          <t>Cumulative adverse childhood experiences and parent-reported allergic conditions and asthma among U.S. children: A nationally representative study.</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>American Psychologist</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000910?dgcid=rss_sd_all</t>
+          <t>https://psycnet.apa.org/record/2027-88271-001</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -4495,22 +4495,22 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>education_learning</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>People underestimate how receptive other people are to different political opinions</t>
+          <t>Associative learning explains “intuitive statistics” in animals.</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Psychological Review</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000727?dgcid=rss_sd_all</t>
+          <t>https://psycnet.apa.org/record/2027-87718-001</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -4537,17 +4537,17 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>On the politicization and polarization of psychology: What psychologists can learn from psychologists</t>
+          <t>A reciprocal model of practice and skill: Navigating between dropout and expertise.</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Psychological Review</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000709?dgcid=rss_sd_all</t>
+          <t>https://psycnet.apa.org/record/2027-87672-001</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -4569,12 +4569,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>gender_equality</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Not all stimuli are conditioned equal – Larger evaluative conditioning effects for fluent stimuli</t>
+          <t>“Friend or foe?” the ironic effect of speaking the minority's language in intergroup conflicts: Palestinian reactions to Jewish-Israelis using Arabic</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -4584,7 +4584,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S002210312600048X?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000739?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>equal</t>
+          <t>friend</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Multiculturalism shapes moral judgments of sexist men across religious groups</t>
+          <t>When it is important to be more virtuous: Cultural tightness exacerbates moral superiority</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000703?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000971?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -4648,17 +4648,17 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>More is more, or is there more to it? Frequency moderations in evaluative conditioning depend on variation in the unconditioned stimuli</t>
+          <t>Visual liking as sensory valuation</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000405?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000928?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -4685,17 +4685,17 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Minority report: How minorities' awareness of power asymmetry drives strategic preparation in opinion debates</t>
+          <t>Visual art and flourishing: Current evidence and emerging directions</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000570?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000904?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -4717,12 +4717,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>gender_equality</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Managing threatened identities across everyday situations</t>
+          <t>Underestimating sexism: Is gender categorization key?</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000363?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126001034?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t/>
+          <t>gender</t>
         </is>
       </c>
     </row>
@@ -4754,22 +4754,22 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>education_learning</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Learning to distrust: One trust experience changes the expected value of trust</t>
+          <t>The sweet spot of seeing: A categorization-based account of visual aesthetic pleasure</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000600?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000898?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -4796,17 +4796,17 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Just a means to an end? Individuals support direct democracy instrumentally, irrespective of conspiracy mentality</t>
+          <t>The psychology of negotiation alternatives: Power, pathways, and performance</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000351?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000953?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Is it my fault? How attributing exclusion to norm violations triggers self-directed emotions</t>
+          <t>Testing the psychological distinctiveness of proscriptive and prescriptive moral norms: A replication and extension of Janoff-Bulman et al. (2009)</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -4843,7 +4843,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000909?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000776?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -4860,17 +4860,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>reject</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Is a random human peer better than a highly supportive chatbot in reducing loneliness over time?</t>
+          <t>Stimulus-category confounds reduce, but do not explain, different roles of intent across moral domains: Valid statistical inference helps explain ‘inconsistent’ findings</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -4880,17 +4880,17 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000417?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126001022?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t/>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>loneliness</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -4902,12 +4902,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>education_learning</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Interpersonal synchrony modulates explicit and implicit self-other blurring: Evidence from an IAT</t>
+          <t>Selective traits and general rewards: Differentiating learning effects on social impression and choice</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000673?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000983?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -4927,7 +4927,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>interpersonal</t>
+          <t>social</t>
         </is>
       </c>
     </row>
@@ -4939,12 +4939,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>mind_acceptance</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Incentivization very weakly improves theory of mind: A multi-sample investigation and meta-analysis</t>
+          <t>Selective ignorance? The role of the information target in allocation decisions</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000260?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000892?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -4976,12 +4976,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>consumer_marketing</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Hypocrisy either way: Judgments of moral actors who choose between conflicting commitments</t>
+          <t>Seeing oneself in the feed: Racialized targeting in food marketing and its impact on adolescents' visual interest and unhealthy food preferences</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000752?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000934?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Holiday greeting inclusivity in organizations: The more the merrier</t>
+          <t>Replication and extension of Carlson and Zaki (2018): Do lay theories of altruism apply equally to all actors?</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000624?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000995?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -5055,17 +5055,17 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Gossip or confrontation? Sanctioning environmental norm violations and the reputation of punishers</t>
+          <t>Racialized Psychotherapy: Understudied Risks and the Case for Empirical Scrutiny</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000454?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000941?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -5092,17 +5092,17 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Giving women credit where credit is due: The role of amplifying, attributing, and appropriating others' ideas</t>
+          <t>Post-negotiation behavior and attitudes: We have a deal, now what?</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000740?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000965?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -5124,22 +5124,22 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Fairness matters: The impact of leaders' emotional expressions on subordinates' behavior</t>
+          <t>Politics in psychiatry and psychotherapis in Japan with personal reflection; Is cognitive behavior therapy non-political?</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000879?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000874?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -5149,7 +5149,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Expectations of middle school children's academic performance in STEM and the Humanities: The effects of genetic and environmental frameworks</t>
+          <t>Persuasion via intermediaries: The pull of extremity</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -5176,7 +5176,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000764?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000910?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -5198,12 +5198,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>emotional_social</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Emotional cues to group hierarchy: Inferences about dominance- versus prestige-based hierarchies from members' emotional expressions</t>
+          <t>People underestimate how receptive other people are to different political opinions</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -5213,7 +5213,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000612?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000727?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -5235,12 +5235,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Editorial Board</t>
+          <t>People feel but don't tell: Dispositional honesty and emotional responses to others' (mis)fortunes</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -5250,7 +5250,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S002210312600082X?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S002210312600096X?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t/>
+          <t>emotional</t>
         </is>
       </c>
     </row>
@@ -5277,17 +5277,17 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Does ignorance love company? The social dynamics of information avoidance</t>
+          <t>Mobile eye-tracking in art museums: From visitor research to museum practice</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000478?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000989?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -5297,7 +5297,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Does attending to the nose vs. eyes reduce the cross-race recognition deficit? A systematic test</t>
+          <t>Is it my fault? How attributing exclusion to norm violations triggers self-directed emotions</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -5324,7 +5324,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000880?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000909?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -5351,17 +5351,17 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Does Behavioral Parent Training Benefit from Cultural Adaptations? A Critical Analysis</t>
+          <t>Is comedy funnier when it is easier to process? The interplay of fluency and coherence in humor appreciation</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Journal of Experimental Social Psychology</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000862?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126001009?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -5388,7 +5388,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Diversity, equity, and inclusion regression: Perceptions of organizations that fail to persevere in their stated commitments</t>
+          <t>Hypocrisy either way: Judgments of moral actors who choose between conflicting commitments</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000946?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000752?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -5420,12 +5420,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>gender_equality</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Decision strategy and perceived humanness: The roles of decision context and decision outcome</t>
+          <t>How and why the omission bias affects victims' and third parties' responses to interpersonal transgressions</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000582?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126001010?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t/>
+          <t>interpersonal</t>
         </is>
       </c>
     </row>
@@ -5457,22 +5457,22 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Critical social justice and its cognitive distortions: Diagnosing the Liberal’s poor mental health</t>
+          <t>Giving women credit where credit is due: The role of amplifying, attributing, and appropriating others' ideas</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Journal of Experimental Social Psychology</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000667?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000740?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>social, mental health</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -5494,22 +5494,22 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>governance_society</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Corrigendum to “A trust inoculation to protect public support of governmentally mandated actions to mitigate climate change” [Journal of Experimental Social Psychology 115 (2024) 104656]</t>
+          <t>From collective guilt to moral implication in collective memory studies</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000442?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X2600093X?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -5519,7 +5519,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>social</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -5531,22 +5531,22 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional_social</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Contemporary antisemitism: Implications for cognitive behavioral therapy</t>
+          <t>Fairness matters: The impact of leaders' emotional expressions on subordinates' behavior</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Journal of Experimental Social Psychology</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000825?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000879?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -5556,7 +5556,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t/>
+          <t>emotional</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Common = ineffective? A replication attempt of the normative dilution effect in the context of political apologies</t>
+          <t>Expectations of middle school children's academic performance in STEM and the Humanities: The effects of genetic and environmental frameworks</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000685?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000764?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Collective streaks motivate prosocial behavior</t>
+          <t>Editorial Board</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000715?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126001083?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -5647,17 +5647,17 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Cognitive conflict in willful ignorance: A mouse-tracking study</t>
+          <t>Does behavioral parent training benefit from cultural adaptations? A critical analysis</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000922?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000862?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -5684,17 +5684,17 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Can cognitive behavioral therapy be value-free and politically neutral?</t>
+          <t>Does attending to the nose vs. eyes reduce the cross-race recognition deficit? A systematic test</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Journal of Experimental Social Psychology</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000655?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000880?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Beyond morality primacy: Inference of competence takes the lead in spontaneous impressions</t>
+          <t>Do people think I'm late in life? An intersubjective approach to culture and the optimal timing of life</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000661?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126001137?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -5758,7 +5758,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Beyond confronting: Cultivating inclusion through proactive Allyship</t>
+          <t>Diversity, equity, and inclusion regression: Perceptions of organizations that fail to persevere in their stated commitments</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000533?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000946?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -5790,12 +5790,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>governance_society</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Beliefs versus reality: People overestimate the actual dishonesty of others</t>
+          <t>Corrigendum to “A trust inoculation to protect public support of governmentally mandated actions to mitigate climate change” [Journal of Experimental Social Psychology 115 (2024) 104656]</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S002210312600034X?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000442?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -5815,7 +5815,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t/>
+          <t>social</t>
         </is>
       </c>
     </row>
@@ -5832,17 +5832,17 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Approach-avoidance action tendencies: A replicable approach/avoidance compatibility effect can be found when valence is task irrelevant</t>
+          <t>Contemporary antisemitism: Implications for cognitive behavioral therapy</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Journal of Experimental Social Psychology</t>
+          <t>Current Opinion in Psychology</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000466?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000825?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -5864,22 +5864,22 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>health_mental_health</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Antisemitism in Professional Clinical Psychology Training</t>
+          <t>Collective streaks motivate prosocial behavior</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Journal of Experimental Social Psychology</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000850?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000715?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -5906,17 +5906,17 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>An intergroup perspective on evolutionary scepticism</t>
+          <t>Cognitive conflict in willful ignorance: A mouse-tracking study</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Current Opinion in Psychology</t>
+          <t>Journal of Experimental Social Psychology</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000849?dgcid=rss_sd_all</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126000922?dgcid=rss_sd_all</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -5943,25 +5943,99 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Against the racialization of reason: Science as a universal method of problem-solving</t>
+          <t>Between law and conscience: Act legality shapes moral evaluation</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
+          <t>Journal of Experimental Social Psychology</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/pii/S0022103126001149?dgcid=rss_sd_all</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>reject</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>health_mental_health</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Antisemitism in professional clinical psychology training</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
           <t>Current Opinion in Psychology</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000679?dgcid=rss_sd_all</t>
-        </is>
-      </c>
-      <c r="F161" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G161" t="inlineStr">
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000850?dgcid=rss_sd_all</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>reject</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Aesthetic Insights from Infant Looking.</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Current Opinion in Psychology</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352250X26000977?dgcid=rss_sd_all</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>